<commit_message>
docs: add contributor guide and refresh unemployment figure
</commit_message>
<xml_diff>
--- a/analysis/econometrics_outputs/Graficos/data_quality/epa_vs_sepe_unemployment_quarterly.xlsx
+++ b/analysis/econometrics_outputs/Graficos/data_quality/epa_vs_sepe_unemployment_quarterly.xlsx
@@ -494,7 +494,7 @@
         <v>8250</v>
       </c>
       <c r="D4" t="n">
-        <v>3316943.666666667</v>
+        <v>3336071.666666667</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -513,7 +513,7 @@
         <v>7663</v>
       </c>
       <c r="D5" t="n">
-        <v>3181886.333333333</v>
+        <v>3181886.666666667</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -570,7 +570,7 @@
         <v>7163</v>
       </c>
       <c r="D8" t="n">
-        <v>2911993</v>
+        <v>2916657</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
@@ -627,7 +627,7 @@
         <v>6666</v>
       </c>
       <c r="D11" t="n">
-        <v>2738612</v>
+        <v>2738774</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
@@ -646,7 +646,7 @@
         <v>6574</v>
       </c>
       <c r="D12" t="n">
-        <v>2696878.666666667</v>
+        <v>2701014</v>
       </c>
       <c r="E12" t="n">
         <v>3</v>
@@ -722,7 +722,7 @@
         <v>5974</v>
       </c>
       <c r="D16" t="n">
-        <v>2565340.333333333</v>
+        <v>2565881</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
@@ -760,7 +760,7 @@
         <v>6168</v>
       </c>
       <c r="D18" t="n">
-        <v>2590842.333333333</v>
+        <v>2591010</v>
       </c>
       <c r="E18" t="n">
         <v>3</v>
@@ -798,7 +798,7 @@
         <v>5311</v>
       </c>
       <c r="D20" t="n">
-        <v>2410477.666666667</v>
+        <v>2417594</v>
       </c>
       <c r="E20" t="n">
         <v>3</v>
@@ -817,7 +817,7 @@
         <v>4875</v>
       </c>
       <c r="D21" t="n">
-        <v>2425798.666666667</v>
+        <v>2425799</v>
       </c>
       <c r="E21" t="n">
         <v>3</v>

</xml_diff>